<commit_message>
Add LLM judging and generation consistency workflows
</commit_message>
<xml_diff>
--- a/data/testset_human_feedback.xlsx
+++ b/data/testset_human_feedback.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/quynguyen/Documents/CodingProjects/prebi_v1/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587E50B9-7FC1-FC43-9DC8-3C444BBCD745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D23DA15-C4B8-694F-BE31-C9192D45BA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34560" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="testset_feedback" sheetId="1" r:id="rId1"/>
@@ -1295,11 +1295,32 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{6649D996-6833-C548-BBDE-C83189B87AE7}">
+  <we:reference id="93533c7f-4dc5-468f-aba4-1c008e1a7ac8" version="1.0.0.8" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200003101" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="2" max="2" width="65.1640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="94.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1307,7 +1328,7 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -1318,29 +1339,29 @@
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="256" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="304" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -1351,7 +1372,7 @@
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -1362,7 +1383,7 @@
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -1373,7 +1394,7 @@
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -1384,7 +1405,7 @@
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -1395,29 +1416,29 @@
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="350" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="365" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -1428,7 +1449,7 @@
       <c r="A12" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -1439,18 +1460,18 @@
       <c r="A13" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>37</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="365" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -1461,18 +1482,18 @@
       <c r="A15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="335" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C16" s="3" t="s">
@@ -1483,7 +1504,7 @@
       <c r="A17" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>49</v>
       </c>
       <c r="C17" s="3" t="s">
@@ -1494,7 +1515,7 @@
       <c r="A18" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="3" t="s">
@@ -1505,7 +1526,7 @@
       <c r="A19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C19" s="3" t="s">
@@ -1516,40 +1537,40 @@
       <c r="A20" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>57</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="208" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>60</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="320" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>63</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="256" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="3" t="s">
         <v>66</v>
       </c>
       <c r="C23" s="3" t="s">

</xml_diff>